<commit_message>
Replace row 4 (Wes Wagner) with verified Scott Rose / ScottWorld
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138sQqZ89s5HQxGgyoe9TcP
</commit_message>
<xml_diff>
--- a/sample/eryk_airtable_VERIFIED.xlsx
+++ b/sample/eryk_airtable_VERIFIED.xlsx
@@ -432,12 +432,12 @@
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -651,52 +651,52 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Wes Wagner</t>
+          <t>Scott Rose</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rarely Decaf</t>
+          <t>ScottWorld</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Founder / Consultant</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Custom apps + automation for service businesses</t>
+          <t>Airtable systems + automation &amp; integrations</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Airtable, Make, Stacker, Xano</t>
+          <t>Airtable, Make, Fillout, Documint</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Solo / small</t>
+          <t>Solo</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Indianapolis, USA</t>
+          <t>Los Angeles, USA</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://westonwagner.com</t>
+          <t>https://www.scottworld.com</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/westonwagner/</t>
+          <t>https://www.linkedin.com/in/scotty321/</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Website verified live; Airtable since 2016; SMB ops automation</t>
+          <t>Website verified live; solo (works directly with clients); Certified Make Partner; one of the original 10 Airtable consultants</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove Team Size column from Eryk verified sample
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138sQqZ89s5HQxGgyoe9TcP
</commit_message>
<xml_diff>
--- a/sample/eryk_airtable_VERIFIED.xlsx
+++ b/sample/eryk_airtable_VERIFIED.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -433,11 +433,10 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,25 +467,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Team Size</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Website</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>LinkedIn URL</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>LinkedIn URL</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -520,25 +514,20 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Solo</t>
+          <t>Udine, Italy</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Udine, Italy</t>
+          <t>https://moninosolutions.com</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://moninosolutions.com</t>
+          <t>https://www.linkedin.com/in/alessio-monino-052518171/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/alessio-monino-052518171/</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
         <is>
           <t>Website verified live; 200+ Airtable projects; #1 Airtable Consultant on Upwork</t>
         </is>
@@ -572,25 +561,20 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Solo</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>https://www.fortmanconsulting.com</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.fortmanconsulting.com</t>
+          <t>https://www.linkedin.com/in/colefortman/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/colefortman/</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
         <is>
           <t>Website verified live; no-code agency + coaching; Zapier Certified</t>
         </is>
@@ -624,25 +608,20 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Solo</t>
+          <t>Belgium (French)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Belgium (French)</t>
+          <t>https://airtable.florianverdonck.be</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://airtable.florianverdonck.be</t>
+          <t>https://www.linkedin.com/in/florianverdonck</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/florianverdonck</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
         <is>
           <t>Website verified live; 120+ Airtable missions; educator</t>
         </is>
@@ -676,25 +655,20 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Solo</t>
+          <t>Los Angeles, USA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Los Angeles, USA</t>
+          <t>https://www.scottworld.com</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.scottworld.com</t>
+          <t>https://www.linkedin.com/in/scotty321/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/scotty321/</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
         <is>
           <t>Website verified live; solo (works directly with clients); Certified Make Partner; one of the original 10 Airtable consultants</t>
         </is>
@@ -728,25 +702,20 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Solo</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>https://allialosa.com</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://allialosa.com</t>
+          <t>https://www.linkedin.com/in/allialosa/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/allialosa/</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
         <is>
           <t>Website verified live; Airtable Community leader; BuiltOnAir co-host</t>
         </is>

</xml_diff>